<commit_message>
Refresh universe gaps — derive pass fills 32,027 cells
Ran the gap-refresh chain on the terminal master:
- fdb_sector_hydrate: sector/industry already maxed (remaining gaps
  are names FinanceDatabase itself lacks — structural, not fixable).
- derive_missing_columns: +32,027 cells from existing inputs —
  fcf_per_share 3.7k -> 24.6k (+20,909), net_cash_pct_mcap +2,927,
  ev_revenue +2,210, cash_pct_mcap +1,781, cash_pct_ev +1,649,
  net_cash +1,538, ev_ebit +642, asset_turnover / pretax_margin /
  eps_diluted +others.
- fill_asymmetry_gaps + re-enrich + archetype_tags + re-enrich.

Multi-archetype names rose 6,469 -> 6,521 as the fuller cash/EV
coverage lets more names qualify. All 8 workbooks regenerated;
verified 0 nan/inf cells, all builders rc=0, Harvard aesthetic intact.

Remaining gaps are legitimate: p_e sparse for loss-makers (no valid
PE), capital_return/buyback_yield EDGAR-only (US filers),
dividend_yield absent for non-payers.
</commit_message>
<xml_diff>
--- a/segment_detail_book.xlsx
+++ b/segment_detail_book.xlsx
@@ -8918,12 +8918,12 @@
       </c>
       <c r="B114" s="14" t="inlineStr">
         <is>
-          <t>COSO</t>
+          <t>SIEB</t>
         </is>
       </c>
       <c r="C114" s="15" t="inlineStr">
         <is>
-          <t>CoastalSouth Bancshares, Inc.</t>
+          <t>Siebert Financial Corp.</t>
         </is>
       </c>
       <c r="D114" s="16" t="inlineStr">
@@ -8937,7 +8937,7 @@
         </is>
       </c>
       <c r="F114" s="18" t="n">
-        <v>326702400</v>
+        <v>69599592</v>
       </c>
       <c r="G114" s="19" t="inlineStr">
         <is>
@@ -8949,43 +8949,53 @@
           <t>–</t>
         </is>
       </c>
-      <c r="I114" s="20" t="n">
-        <v>12.204545</v>
-      </c>
-      <c r="J114" s="22" t="n">
-        <v>-21.25150433941449</v>
-      </c>
-      <c r="K114" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="I114" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J114" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K114" s="22" t="n">
+        <v>5.17888936540735</v>
       </c>
       <c r="L114" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M114" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>7.23199371130981</v>
+      </c>
+      <c r="M114" s="20" t="n">
+        <v>-1.897588315217392</v>
       </c>
       <c r="N114" s="22" t="n">
-        <v>26.10063202591439</v>
+        <v>-64.87603317998357</v>
       </c>
       <c r="O114" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P114" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q114" s="15" t="n"/>
-      <c r="R114" s="17" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="P114" s="20" t="n">
+        <v>0.9865046689171856</v>
+      </c>
+      <c r="Q114" s="15" t="inlineStr">
+        <is>
+          <t>Financial Services (99%)</t>
+        </is>
+      </c>
+      <c r="R114" s="17" t="inlineStr">
+        <is>
+          <t>Financial Services 99%; Media Sports And Entertainment 1%</t>
+        </is>
+      </c>
       <c r="S114" s="18" t="n">
         <v>0</v>
       </c>
       <c r="T114" s="17" t="n"/>
-      <c r="U114" s="15" t="n"/>
+      <c r="U114" s="15" t="inlineStr">
+        <is>
+          <t>Financial Services +11%</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="13" t="n">
@@ -8993,12 +9003,12 @@
       </c>
       <c r="B115" s="14" t="inlineStr">
         <is>
-          <t>GENC</t>
+          <t>COSO</t>
         </is>
       </c>
       <c r="C115" s="15" t="inlineStr">
         <is>
-          <t>Gencor Industries, Inc.</t>
+          <t>CoastalSouth Bancshares, Inc.</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -9008,37 +9018,43 @@
       </c>
       <c r="E115" s="17" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F115" s="18" t="n">
-        <v>222503920</v>
+        <v>326702400</v>
       </c>
       <c r="G115" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H115" s="20" t="n">
-        <v>5.414</v>
+      <c r="H115" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="I115" s="20" t="n">
-        <v>17.056181</v>
+        <v>12.204545</v>
       </c>
       <c r="J115" s="22" t="n">
-        <v>10.74008646076678</v>
-      </c>
-      <c r="K115" s="22" t="n">
-        <v>9.653633066284021</v>
+        <v>-21.25150433941449</v>
+      </c>
+      <c r="K115" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L115" s="22" t="n">
-        <v>13.72795033364932</v>
-      </c>
-      <c r="M115" s="20" t="n">
-        <v>-9.984835149955996</v>
+        <v>0</v>
+      </c>
+      <c r="M115" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N115" s="22" t="n">
-        <v>3.9158808074461</v>
+        <v>26.10063202591439</v>
       </c>
       <c r="O115" s="18" t="n">
         <v>0</v>
@@ -9062,12 +9078,12 @@
       </c>
       <c r="B116" s="14" t="inlineStr">
         <is>
-          <t>CRMD</t>
+          <t>GENC</t>
         </is>
       </c>
       <c r="C116" s="15" t="inlineStr">
         <is>
-          <t>CorMedix Inc.</t>
+          <t>Gencor Industries, Inc.</t>
         </is>
       </c>
       <c r="D116" s="16" t="inlineStr">
@@ -9077,37 +9093,37 @@
       </c>
       <c r="E116" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F116" s="18" t="n">
-        <v>615847296</v>
-      </c>
-      <c r="G116" s="24" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+        <v>222503920</v>
+      </c>
+      <c r="G116" s="19" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="H116" s="20" t="n">
-        <v>2.558</v>
+        <v>5.414</v>
       </c>
       <c r="I116" s="20" t="n">
-        <v>3.6175113</v>
+        <v>17.056181</v>
       </c>
       <c r="J116" s="22" t="n">
-        <v>10.76033467943529</v>
+        <v>10.74008646076678</v>
       </c>
       <c r="K116" s="22" t="n">
-        <v>59.72797205767642</v>
+        <v>9.653633066284021</v>
       </c>
       <c r="L116" s="22" t="n">
-        <v>53.68693204238568</v>
+        <v>13.72795033364932</v>
       </c>
       <c r="M116" s="20" t="n">
-        <v>0.0022886577129476</v>
+        <v>-9.984835149955996</v>
       </c>
       <c r="N116" s="22" t="n">
-        <v>-35.4148805667681</v>
+        <v>3.9158808074461</v>
       </c>
       <c r="O116" s="18" t="n">
         <v>0</v>
@@ -9131,12 +9147,12 @@
       </c>
       <c r="B117" s="14" t="inlineStr">
         <is>
-          <t>SMID</t>
+          <t>CRMD</t>
         </is>
       </c>
       <c r="C117" s="15" t="inlineStr">
         <is>
-          <t>Smith-Midland Corporation</t>
+          <t>CorMedix Inc.</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -9146,11 +9162,11 @@
       </c>
       <c r="E117" s="17" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F117" s="18" t="n">
-        <v>157869984</v>
+        <v>615847296</v>
       </c>
       <c r="G117" s="24" t="inlineStr">
         <is>
@@ -9158,25 +9174,25 @@
         </is>
       </c>
       <c r="H117" s="20" t="n">
-        <v>8.513999999999999</v>
+        <v>2.558</v>
       </c>
       <c r="I117" s="20" t="n">
-        <v>15.025252</v>
+        <v>3.6175113</v>
       </c>
       <c r="J117" s="22" t="n">
-        <v>-1.33140004307622</v>
+        <v>10.76033467943529</v>
       </c>
       <c r="K117" s="22" t="n">
-        <v>23.5026343072573</v>
+        <v>59.72797205767642</v>
       </c>
       <c r="L117" s="22" t="n">
-        <v>21.55148427969094</v>
+        <v>53.68693204238568</v>
       </c>
       <c r="M117" s="20" t="n">
-        <v>-0.3648145389542678</v>
+        <v>0.0022886577129476</v>
       </c>
       <c r="N117" s="22" t="n">
-        <v>-5.50939003710083</v>
+        <v>-35.4148805667681</v>
       </c>
       <c r="O117" s="18" t="n">
         <v>0</v>
@@ -9200,12 +9216,12 @@
       </c>
       <c r="B118" s="14" t="inlineStr">
         <is>
-          <t>TRST</t>
+          <t>SMID</t>
         </is>
       </c>
       <c r="C118" s="15" t="inlineStr">
         <is>
-          <t>TrustCo Bank Corp NY</t>
+          <t>Smith-Midland Corporation</t>
         </is>
       </c>
       <c r="D118" s="16" t="inlineStr">
@@ -9215,43 +9231,37 @@
       </c>
       <c r="E118" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="F118" s="18" t="n">
-        <v>955173248</v>
-      </c>
-      <c r="G118" s="19" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
-        </is>
-      </c>
-      <c r="H118" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>157869984</v>
+      </c>
+      <c r="G118" s="24" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="H118" s="20" t="n">
+        <v>8.513999999999999</v>
       </c>
       <c r="I118" s="20" t="n">
-        <v>16.029325</v>
+        <v>15.025252</v>
       </c>
       <c r="J118" s="22" t="n">
-        <v>5.41001892070669</v>
-      </c>
-      <c r="K118" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>-1.33140004307622</v>
+      </c>
+      <c r="K118" s="22" t="n">
+        <v>23.5026343072573</v>
       </c>
       <c r="L118" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M118" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>21.55148427969094</v>
+      </c>
+      <c r="M118" s="20" t="n">
+        <v>-0.3648145389542678</v>
       </c>
       <c r="N118" s="22" t="n">
-        <v>54.78020860532192</v>
+        <v>-5.50939003710083</v>
       </c>
       <c r="O118" s="18" t="n">
         <v>0</v>
@@ -9275,12 +9285,12 @@
       </c>
       <c r="B119" s="14" t="inlineStr">
         <is>
-          <t>QTWO</t>
+          <t>TRST</t>
         </is>
       </c>
       <c r="C119" s="15" t="inlineStr">
         <is>
-          <t>Q2 Holdings, Inc.</t>
+          <t>TrustCo Bank Corp NY</t>
         </is>
       </c>
       <c r="D119" s="16" t="inlineStr">
@@ -9290,37 +9300,43 @@
       </c>
       <c r="E119" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F119" s="18" t="n">
-        <v>2999186432</v>
-      </c>
-      <c r="G119" s="24" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="H119" s="20" t="n">
-        <v>30.444</v>
+        <v>955173248</v>
+      </c>
+      <c r="G119" s="19" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
+        </is>
+      </c>
+      <c r="H119" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="I119" s="20" t="n">
-        <v>42.39823</v>
+        <v>16.029325</v>
       </c>
       <c r="J119" s="22" t="n">
-        <v>3.71867384690194</v>
-      </c>
-      <c r="K119" s="22" t="n">
-        <v>18.83167993346798</v>
+        <v>5.41001892070669</v>
+      </c>
+      <c r="K119" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L119" s="22" t="n">
-        <v>16.52474500352978</v>
-      </c>
-      <c r="M119" s="20" t="n">
-        <v>-0.2577192775699007</v>
+        <v>0</v>
+      </c>
+      <c r="M119" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N119" s="22" t="n">
-        <v>-47.170678900731</v>
+        <v>54.78020860532192</v>
       </c>
       <c r="O119" s="18" t="n">
         <v>0</v>
@@ -9344,12 +9360,12 @@
       </c>
       <c r="B120" s="14" t="inlineStr">
         <is>
-          <t>SUNE</t>
+          <t>QTWO</t>
         </is>
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>SUNation Energy Inc. Common St</t>
+          <t>Q2 Holdings, Inc.</t>
         </is>
       </c>
       <c r="D120" s="16" t="inlineStr">
@@ -9359,63 +9375,53 @@
       </c>
       <c r="E120" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Communication </t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F120" s="18" t="n">
-        <v>10143001</v>
-      </c>
-      <c r="G120" s="19" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+        <v>2999186432</v>
+      </c>
+      <c r="G120" s="24" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="H120" s="20" t="n">
-        <v>-1.219154062695544</v>
+        <v>30.444</v>
       </c>
       <c r="I120" s="20" t="n">
-        <v>0.024325127</v>
+        <v>42.39823</v>
       </c>
       <c r="J120" s="22" t="n">
-        <v>-202.6520054738409</v>
+        <v>3.71867384690194</v>
       </c>
       <c r="K120" s="22" t="n">
-        <v>-35.17300762638625</v>
+        <v>18.83167993346798</v>
       </c>
       <c r="L120" s="22" t="n">
-        <v>-9.68347120242926</v>
+        <v>16.52474500352978</v>
       </c>
       <c r="M120" s="20" t="n">
-        <v>-0.4118934629871731</v>
+        <v>-0.2577192775699007</v>
       </c>
       <c r="N120" s="22" t="n">
-        <v>-19.51219441279421</v>
+        <v>-47.170678900731</v>
       </c>
       <c r="O120" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="P120" s="20" t="n">
-        <v>0.5750863857690269</v>
-      </c>
-      <c r="Q120" s="15" t="inlineStr">
-        <is>
-          <t>Sunation NY (69%)</t>
-        </is>
-      </c>
-      <c r="R120" s="17" t="inlineStr">
-        <is>
-          <t>Sunation NY 69%; Hawaii Energy Connection 31%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P120" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q120" s="15" t="n"/>
+      <c r="R120" s="17" t="n"/>
       <c r="S120" s="18" t="n">
         <v>0</v>
       </c>
       <c r="T120" s="17" t="n"/>
-      <c r="U120" s="15" t="inlineStr">
-        <is>
-          <t>Hawaii Energy Connec +30%</t>
-        </is>
-      </c>
+      <c r="U120" s="15" t="n"/>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="13" t="n">
@@ -9423,12 +9429,12 @@
       </c>
       <c r="B121" s="14" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>SUNE</t>
         </is>
       </c>
       <c r="C121" s="15" t="inlineStr">
         <is>
-          <t>Freshworks Inc. Class A Common</t>
+          <t>SUNation Energy Inc. Common St</t>
         </is>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -9438,11 +9444,11 @@
       </c>
       <c r="E121" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t xml:space="preserve">Communication </t>
         </is>
       </c>
       <c r="F121" s="18" t="n">
-        <v>2722876672</v>
+        <v>10143001</v>
       </c>
       <c r="G121" s="19" t="inlineStr">
         <is>
@@ -9450,45 +9456,51 @@
         </is>
       </c>
       <c r="H121" s="20" t="n">
-        <v>57.225</v>
+        <v>-1.219154062695544</v>
       </c>
       <c r="I121" s="20" t="n">
-        <v>16.147541</v>
+        <v>0.024325127</v>
       </c>
       <c r="J121" s="22" t="n">
-        <v>8.84784932596617</v>
+        <v>-202.6520054738409</v>
       </c>
       <c r="K121" s="22" t="n">
-        <v>5.582241290864149</v>
+        <v>-35.17300762638625</v>
       </c>
       <c r="L121" s="22" t="n">
-        <v>4.92682820440121</v>
+        <v>-9.68347120242926</v>
       </c>
       <c r="M121" s="20" t="n">
-        <v>-17.25127559935696</v>
+        <v>-0.4118934629871731</v>
       </c>
       <c r="N121" s="22" t="n">
-        <v>-37.93574946904199</v>
+        <v>-19.51219441279421</v>
       </c>
       <c r="O121" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P121" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q121" s="15" t="n"/>
-      <c r="R121" s="17" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="P121" s="20" t="n">
+        <v>0.5750863857690269</v>
+      </c>
+      <c r="Q121" s="15" t="inlineStr">
+        <is>
+          <t>Sunation NY (69%)</t>
+        </is>
+      </c>
+      <c r="R121" s="17" t="inlineStr">
+        <is>
+          <t>Sunation NY 69%; Hawaii Energy Connection 31%</t>
+        </is>
+      </c>
       <c r="S121" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="T121" s="17" t="inlineStr">
-        <is>
-          <t>North America 30%; US 27%; EMEA 25%</t>
-        </is>
-      </c>
-      <c r="U121" s="15" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="T121" s="17" t="n"/>
+      <c r="U121" s="15" t="inlineStr">
+        <is>
+          <t>Hawaii Energy Connec +30%</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="13" t="n">
@@ -9496,12 +9508,12 @@
       </c>
       <c r="B122" s="14" t="inlineStr">
         <is>
-          <t>WSFS</t>
+          <t>FRSH</t>
         </is>
       </c>
       <c r="C122" s="15" t="inlineStr">
         <is>
-          <t>WSFS Financial Corporation</t>
+          <t>Freshworks Inc. Class A Common</t>
         </is>
       </c>
       <c r="D122" s="16" t="inlineStr">
@@ -9511,69 +9523,57 @@
       </c>
       <c r="E122" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F122" s="18" t="n">
-        <v>4026127616</v>
+        <v>2722876672</v>
       </c>
       <c r="G122" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H122" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H122" s="20" t="n">
+        <v>57.225</v>
       </c>
       <c r="I122" s="20" t="n">
-        <v>13.789661</v>
+        <v>16.147541</v>
       </c>
       <c r="J122" s="22" t="n">
-        <v>6.158366732153779</v>
-      </c>
-      <c r="K122" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>8.84784932596617</v>
+      </c>
+      <c r="K122" s="22" t="n">
+        <v>5.582241290864149</v>
       </c>
       <c r="L122" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M122" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>4.92682820440121</v>
+      </c>
+      <c r="M122" s="20" t="n">
+        <v>-17.25127559935696</v>
       </c>
       <c r="N122" s="22" t="n">
-        <v>37.01048893948796</v>
+        <v>-37.93574946904199</v>
       </c>
       <c r="O122" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="P122" s="20" t="n">
-        <v>0.5461404223281471</v>
-      </c>
-      <c r="Q122" s="15" t="inlineStr">
-        <is>
-          <t>Wsfs Bank (70%)</t>
-        </is>
-      </c>
-      <c r="R122" s="17" t="inlineStr">
-        <is>
-          <t>Wsfs Bank 70%; Wealth Management 22%; Cash Connect 8%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P122" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q122" s="15" t="n"/>
+      <c r="R122" s="17" t="n"/>
       <c r="S122" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T122" s="17" t="n"/>
-      <c r="U122" s="15" t="inlineStr">
-        <is>
-          <t>Wealth Management +15%</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="T122" s="17" t="inlineStr">
+        <is>
+          <t>North America 30%; US 27%; EMEA 25%</t>
+        </is>
+      </c>
+      <c r="U122" s="15" t="n"/>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="13" t="n">
@@ -9581,12 +9581,12 @@
       </c>
       <c r="B123" s="14" t="inlineStr">
         <is>
-          <t>RXST</t>
+          <t>WSFS</t>
         </is>
       </c>
       <c r="C123" s="15" t="inlineStr">
         <is>
-          <t>RxSight Inc. Common Stock</t>
+          <t>WSFS Financial Corporation</t>
         </is>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -9596,55 +9596,69 @@
       </c>
       <c r="E123" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F123" s="18" t="n">
-        <v>221885824</v>
+        <v>4026127616</v>
       </c>
       <c r="G123" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H123" s="20" t="n">
-        <v>-0.7888837692804765</v>
-      </c>
-      <c r="I123" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H123" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I123" s="20" t="n">
+        <v>13.789661</v>
       </c>
       <c r="J123" s="22" t="n">
-        <v>-8.225567245596439</v>
-      </c>
-      <c r="K123" s="22" t="n">
-        <v>-66.3179452171687</v>
+        <v>6.158366732153779</v>
+      </c>
+      <c r="K123" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L123" s="22" t="n">
-        <v>-26.46713265913147</v>
-      </c>
-      <c r="M123" s="20" t="n">
-        <v>6.099176804427837</v>
+        <v>0</v>
+      </c>
+      <c r="M123" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N123" s="22" t="n">
-        <v>-57.32532194388769</v>
+        <v>37.01048893948796</v>
       </c>
       <c r="O123" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P123" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q123" s="15" t="n"/>
-      <c r="R123" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="P123" s="20" t="n">
+        <v>0.5461404223281471</v>
+      </c>
+      <c r="Q123" s="15" t="inlineStr">
+        <is>
+          <t>Wsfs Bank (70%)</t>
+        </is>
+      </c>
+      <c r="R123" s="17" t="inlineStr">
+        <is>
+          <t>Wsfs Bank 70%; Wealth Management 22%; Cash Connect 8%</t>
+        </is>
+      </c>
       <c r="S123" s="18" t="n">
         <v>0</v>
       </c>
       <c r="T123" s="17" t="n"/>
-      <c r="U123" s="15" t="n"/>
+      <c r="U123" s="15" t="inlineStr">
+        <is>
+          <t>Wealth Management +15%</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="13" t="n">
@@ -9652,12 +9666,12 @@
       </c>
       <c r="B124" s="14" t="inlineStr">
         <is>
-          <t>ACCS</t>
+          <t>RXST</t>
         </is>
       </c>
       <c r="C124" s="15" t="inlineStr">
         <is>
-          <t>ACCESS Newswire Inc. Common St</t>
+          <t>RxSight Inc. Common Stock</t>
         </is>
       </c>
       <c r="D124" s="16" t="inlineStr">
@@ -9667,11 +9681,11 @@
       </c>
       <c r="E124" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Communication </t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F124" s="18" t="n">
-        <v>26553866</v>
+        <v>221885824</v>
       </c>
       <c r="G124" s="19" t="inlineStr">
         <is>
@@ -9679,7 +9693,7 @@
         </is>
       </c>
       <c r="H124" s="20" t="n">
-        <v>20.806</v>
+        <v>-0.7888837692804765</v>
       </c>
       <c r="I124" s="21" t="inlineStr">
         <is>
@@ -9687,19 +9701,19 @@
         </is>
       </c>
       <c r="J124" s="22" t="n">
-        <v>10.91194270159679</v>
+        <v>-8.225567245596439</v>
       </c>
       <c r="K124" s="22" t="n">
-        <v>-6.34942688433483</v>
+        <v>-66.3179452171687</v>
       </c>
       <c r="L124" s="22" t="n">
-        <v>4.30169326672266</v>
+        <v>-26.46713265913147</v>
       </c>
       <c r="M124" s="20" t="n">
-        <v>-0.1562178828365878</v>
+        <v>6.099176804427837</v>
       </c>
       <c r="N124" s="22" t="n">
-        <v>-25.5839796713547</v>
+        <v>-57.32532194388769</v>
       </c>
       <c r="O124" s="18" t="n">
         <v>0</v>
@@ -9723,12 +9737,12 @@
       </c>
       <c r="B125" s="14" t="inlineStr">
         <is>
-          <t>TACT</t>
+          <t>ACCS</t>
         </is>
       </c>
       <c r="C125" s="15" t="inlineStr">
         <is>
-          <t>TransAct Technologies Incorpor</t>
+          <t>ACCESS Newswire Inc. Common St</t>
         </is>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -9738,11 +9752,11 @@
       </c>
       <c r="E125" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t xml:space="preserve">Communication </t>
         </is>
       </c>
       <c r="F125" s="18" t="n">
-        <v>54515660</v>
+        <v>26553866</v>
       </c>
       <c r="G125" s="19" t="inlineStr">
         <is>
@@ -9750,55 +9764,43 @@
         </is>
       </c>
       <c r="H125" s="20" t="n">
-        <v>15.2490059473237</v>
-      </c>
-      <c r="I125" s="20" t="n">
-        <v>55.99555555555556</v>
+        <v>20.806</v>
+      </c>
+      <c r="I125" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J125" s="22" t="n">
-        <v>-10.67708135131403</v>
+        <v>10.91194270159679</v>
       </c>
       <c r="K125" s="22" t="n">
-        <v>3.8075407154012</v>
+        <v>-6.34942688433483</v>
       </c>
       <c r="L125" s="22" t="n">
-        <v>-0.14180264180264</v>
+        <v>4.30169326672266</v>
       </c>
       <c r="M125" s="20" t="n">
-        <v>231.1232876712329</v>
+        <v>-0.1562178828365878</v>
       </c>
       <c r="N125" s="22" t="n">
-        <v>2.28571210588727</v>
+        <v>-25.5839796713547</v>
       </c>
       <c r="O125" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P125" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q125" s="15" t="inlineStr">
-        <is>
-          <t>Transact (100%)</t>
-        </is>
-      </c>
-      <c r="R125" s="17" t="inlineStr">
-        <is>
-          <t>Transact 100%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P125" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q125" s="15" t="n"/>
+      <c r="R125" s="17" t="n"/>
       <c r="S125" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="T125" s="17" t="inlineStr">
-        <is>
-          <t>US 80%; Non Us 20%</t>
-        </is>
-      </c>
-      <c r="U125" s="15" t="inlineStr">
-        <is>
-          <t>Transact +19%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T125" s="17" t="n"/>
+      <c r="U125" s="15" t="n"/>
     </row>
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="13" t="n">
@@ -9806,12 +9808,12 @@
       </c>
       <c r="B126" s="14" t="inlineStr">
         <is>
-          <t>NBBK</t>
+          <t>TACT</t>
         </is>
       </c>
       <c r="C126" s="15" t="inlineStr">
         <is>
-          <t>NB Bancorp Inc. Common Stock</t>
+          <t>TransAct Technologies Incorpor</t>
         </is>
       </c>
       <c r="D126" s="16" t="inlineStr">
@@ -9821,59 +9823,67 @@
       </c>
       <c r="E126" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F126" s="18" t="n">
-        <v>933929408</v>
+        <v>54515660</v>
       </c>
       <c r="G126" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H126" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H126" s="20" t="n">
+        <v>15.2490059473237</v>
       </c>
       <c r="I126" s="20" t="n">
-        <v>15.547444</v>
+        <v>55.99555555555556</v>
       </c>
       <c r="J126" s="22" t="n">
-        <v>6.8259973458476</v>
-      </c>
-      <c r="K126" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>-10.67708135131403</v>
+      </c>
+      <c r="K126" s="22" t="n">
+        <v>3.8075407154012</v>
       </c>
       <c r="L126" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M126" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>-0.14180264180264</v>
+      </c>
+      <c r="M126" s="20" t="n">
+        <v>231.1232876712329</v>
       </c>
       <c r="N126" s="22" t="n">
-        <v>9.52875917003306</v>
+        <v>2.28571210588727</v>
       </c>
       <c r="O126" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P126" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q126" s="15" t="n"/>
-      <c r="R126" s="17" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="P126" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q126" s="15" t="inlineStr">
+        <is>
+          <t>Transact (100%)</t>
+        </is>
+      </c>
+      <c r="R126" s="17" t="inlineStr">
+        <is>
+          <t>Transact 100%</t>
+        </is>
+      </c>
       <c r="S126" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T126" s="17" t="n"/>
-      <c r="U126" s="15" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="T126" s="17" t="inlineStr">
+        <is>
+          <t>US 80%; Non Us 20%</t>
+        </is>
+      </c>
+      <c r="U126" s="15" t="inlineStr">
+        <is>
+          <t>Transact +19%</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="13" t="n">
@@ -9881,12 +9891,12 @@
       </c>
       <c r="B127" s="14" t="inlineStr">
         <is>
-          <t>ACRV</t>
+          <t>NBBK</t>
         </is>
       </c>
       <c r="C127" s="15" t="inlineStr">
         <is>
-          <t>Acrivon Therapeutics Inc. Comm</t>
+          <t>NB Bancorp Inc. Common Stock</t>
         </is>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -9896,39 +9906,43 @@
       </c>
       <c r="E127" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F127" s="18" t="n">
-        <v>71906904</v>
+        <v>933929408</v>
       </c>
       <c r="G127" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H127" s="20" t="n">
-        <v>0.289</v>
-      </c>
-      <c r="I127" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H127" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I127" s="20" t="n">
+        <v>15.547444</v>
       </c>
       <c r="J127" s="22" t="n">
-        <v>-86.23919495512193</v>
-      </c>
-      <c r="K127" s="22" t="n">
-        <v>2505.630026809652</v>
+        <v>6.8259973458476</v>
+      </c>
+      <c r="K127" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L127" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="M127" s="20" t="n">
-        <v>1.400142584402716</v>
+      <c r="M127" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N127" s="22" t="n">
-        <v>60.9090856875271</v>
+        <v>9.52875917003306</v>
       </c>
       <c r="O127" s="18" t="n">
         <v>0</v>
@@ -9952,12 +9966,12 @@
       </c>
       <c r="B128" s="14" t="inlineStr">
         <is>
-          <t>BOOM</t>
+          <t>ACRV</t>
         </is>
       </c>
       <c r="C128" s="15" t="inlineStr">
         <is>
-          <t>DMC Global Inc.</t>
+          <t>Acrivon Therapeutics Inc. Comm</t>
         </is>
       </c>
       <c r="D128" s="16" t="inlineStr">
@@ -9967,11 +9981,11 @@
       </c>
       <c r="E128" s="17" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F128" s="18" t="n">
-        <v>123836296</v>
+        <v>71906904</v>
       </c>
       <c r="G128" s="19" t="inlineStr">
         <is>
@@ -9979,7 +9993,7 @@
         </is>
       </c>
       <c r="H128" s="20" t="n">
-        <v>13.541</v>
+        <v>0.289</v>
       </c>
       <c r="I128" s="21" t="inlineStr">
         <is>
@@ -9987,49 +10001,35 @@
         </is>
       </c>
       <c r="J128" s="22" t="n">
-        <v>8.129076452317911</v>
+        <v>-86.23919495512193</v>
       </c>
       <c r="K128" s="22" t="n">
-        <v>2.69253759150435</v>
+        <v>2505.630026809652</v>
       </c>
       <c r="L128" s="22" t="n">
-        <v>3.75265505975483</v>
+        <v>0</v>
       </c>
       <c r="M128" s="20" t="n">
-        <v>1.020321876704855</v>
+        <v>1.400142584402716</v>
       </c>
       <c r="N128" s="22" t="n">
-        <v>1.0204036947789</v>
+        <v>60.9090856875271</v>
       </c>
       <c r="O128" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="P128" s="20" t="n">
-        <v>0.3822472055915061</v>
-      </c>
-      <c r="Q128" s="15" t="inlineStr">
-        <is>
-          <t>Dyna Energetics (44%)</t>
-        </is>
-      </c>
-      <c r="R128" s="17" t="inlineStr">
-        <is>
-          <t>Dyna Energetics 44%; Arcadia Products 40%; Nobel Clad 15%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P128" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q128" s="15" t="n"/>
+      <c r="R128" s="17" t="n"/>
       <c r="S128" s="18" t="n">
-        <v>21</v>
-      </c>
-      <c r="T128" s="17" t="inlineStr">
-        <is>
-          <t>US 41%; West 33%; Rest Of The World 5%</t>
-        </is>
-      </c>
-      <c r="U128" s="15" t="inlineStr">
-        <is>
-          <t>Arcadia Products -1%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T128" s="17" t="n"/>
+      <c r="U128" s="15" t="n"/>
     </row>
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="13" t="n">
@@ -10037,12 +10037,12 @@
       </c>
       <c r="B129" s="14" t="inlineStr">
         <is>
-          <t>NRIM</t>
+          <t>BOOM</t>
         </is>
       </c>
       <c r="C129" s="15" t="inlineStr">
         <is>
-          <t>Northrim BanCorp, Inc.</t>
+          <t>DMC Global Inc.</t>
         </is>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -10052,67 +10052,67 @@
       </c>
       <c r="E129" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="F129" s="18" t="n">
-        <v>621963648</v>
+        <v>123836296</v>
       </c>
       <c r="G129" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H129" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I129" s="20" t="n">
-        <v>9.708333</v>
+      <c r="H129" s="20" t="n">
+        <v>13.541</v>
+      </c>
+      <c r="I129" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J129" s="22" t="n">
-        <v>7.154905282262169</v>
-      </c>
-      <c r="K129" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>8.129076452317911</v>
+      </c>
+      <c r="K129" s="22" t="n">
+        <v>2.69253759150435</v>
       </c>
       <c r="L129" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M129" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>3.75265505975483</v>
+      </c>
+      <c r="M129" s="20" t="n">
+        <v>1.020321876704855</v>
       </c>
       <c r="N129" s="22" t="n">
-        <v>7.62249350229726</v>
+        <v>1.0204036947789</v>
       </c>
       <c r="O129" s="18" t="n">
         <v>3</v>
       </c>
       <c r="P129" s="20" t="n">
-        <v>0.6090673877493771</v>
+        <v>0.3822472055915061</v>
       </c>
       <c r="Q129" s="15" t="inlineStr">
         <is>
-          <t>Community Banking (76%)</t>
+          <t>Dyna Energetics (44%)</t>
         </is>
       </c>
       <c r="R129" s="17" t="inlineStr">
         <is>
-          <t>Community Banking 76%; Home Mortgage Lending 17%; Specialty Finance 7%</t>
+          <t>Dyna Energetics 44%; Arcadia Products 40%; Nobel Clad 15%</t>
         </is>
       </c>
       <c r="S129" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T129" s="17" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="T129" s="17" t="inlineStr">
+        <is>
+          <t>US 41%; West 33%; Rest Of The World 5%</t>
+        </is>
+      </c>
       <c r="U129" s="15" t="inlineStr">
         <is>
-          <t>Specialty Finance +257%</t>
+          <t>Arcadia Products -1%</t>
         </is>
       </c>
     </row>
@@ -10122,12 +10122,12 @@
       </c>
       <c r="B130" s="14" t="inlineStr">
         <is>
-          <t>PASG</t>
+          <t>NRIM</t>
         </is>
       </c>
       <c r="C130" s="15" t="inlineStr">
         <is>
-          <t>Passage Bio, Inc.</t>
+          <t>Northrim BanCorp, Inc.</t>
         </is>
       </c>
       <c r="D130" s="16" t="inlineStr">
@@ -10137,55 +10137,69 @@
       </c>
       <c r="E130" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F130" s="18" t="n">
-        <v>15100206</v>
+        <v>621963648</v>
       </c>
       <c r="G130" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H130" s="20" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="I130" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H130" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I130" s="20" t="n">
+        <v>9.708333</v>
       </c>
       <c r="J130" s="22" t="n">
-        <v>-188.1721537819593</v>
-      </c>
-      <c r="K130" s="22" t="n">
-        <v>1219.643866591294</v>
+        <v>7.154905282262169</v>
+      </c>
+      <c r="K130" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L130" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="M130" s="20" t="n">
-        <v>0.5254932465879358</v>
+      <c r="M130" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N130" s="22" t="n">
-        <v>-12.12121649988203</v>
+        <v>7.62249350229726</v>
       </c>
       <c r="O130" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P130" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q130" s="15" t="n"/>
-      <c r="R130" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="P130" s="20" t="n">
+        <v>0.6090673877493771</v>
+      </c>
+      <c r="Q130" s="15" t="inlineStr">
+        <is>
+          <t>Community Banking (76%)</t>
+        </is>
+      </c>
+      <c r="R130" s="17" t="inlineStr">
+        <is>
+          <t>Community Banking 76%; Home Mortgage Lending 17%; Specialty Finance 7%</t>
+        </is>
+      </c>
       <c r="S130" s="18" t="n">
         <v>0</v>
       </c>
       <c r="T130" s="17" t="n"/>
-      <c r="U130" s="15" t="n"/>
+      <c r="U130" s="15" t="inlineStr">
+        <is>
+          <t>Specialty Finance +257%</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="13" t="n">
@@ -10193,12 +10207,12 @@
       </c>
       <c r="B131" s="14" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>PASG</t>
         </is>
       </c>
       <c r="C131" s="15" t="inlineStr">
         <is>
-          <t>Rigel Pharmaceuticals, Inc.</t>
+          <t>Passage Bio, Inc.</t>
         </is>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -10212,7 +10226,7 @@
         </is>
       </c>
       <c r="F131" s="18" t="n">
-        <v>715845440</v>
+        <v>15100206</v>
       </c>
       <c r="G131" s="19" t="inlineStr">
         <is>
@@ -10220,51 +10234,43 @@
         </is>
       </c>
       <c r="H131" s="20" t="n">
-        <v>4.842</v>
-      </c>
-      <c r="I131" s="20" t="n">
-        <v>2.0057023</v>
+        <v>0.333</v>
+      </c>
+      <c r="I131" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J131" s="22" t="n">
-        <v>-1.43550383550229</v>
+        <v>-188.1721537819593</v>
       </c>
       <c r="K131" s="22" t="n">
-        <v>27.15453070970258</v>
+        <v>1219.643866591294</v>
       </c>
       <c r="L131" s="22" t="n">
-        <v>43.79434694279223</v>
+        <v>0</v>
       </c>
       <c r="M131" s="20" t="n">
-        <v>0.1557346455313411</v>
+        <v>0.5254932465879358</v>
       </c>
       <c r="N131" s="22" t="n">
-        <v>46.96048918565198</v>
+        <v>-12.12121649988203</v>
       </c>
       <c r="O131" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P131" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q131" s="15" t="inlineStr">
-        <is>
-          <t>Single Reportable (100%)</t>
-        </is>
-      </c>
-      <c r="R131" s="17" t="inlineStr">
-        <is>
-          <t>Single Reportable 100%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P131" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q131" s="15" t="n"/>
+      <c r="R131" s="17" t="n"/>
       <c r="S131" s="18" t="n">
         <v>0</v>
       </c>
       <c r="T131" s="17" t="n"/>
-      <c r="U131" s="15" t="inlineStr">
-        <is>
-          <t>Single Reportable +64%</t>
-        </is>
-      </c>
+      <c r="U131" s="15" t="n"/>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="13" t="n">
@@ -10272,12 +10278,12 @@
       </c>
       <c r="B132" s="14" t="inlineStr">
         <is>
-          <t>CATO</t>
+          <t>RIGL</t>
         </is>
       </c>
       <c r="C132" s="15" t="inlineStr">
         <is>
-          <t>The Cato Corporation</t>
+          <t>Rigel Pharmaceuticals, Inc.</t>
         </is>
       </c>
       <c r="D132" s="16" t="inlineStr">
@@ -10287,11 +10293,11 @@
       </c>
       <c r="E132" s="17" t="inlineStr">
         <is>
-          <t>Consumer Discr</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F132" s="18" t="n">
-        <v>66662584</v>
+        <v>715845440</v>
       </c>
       <c r="G132" s="19" t="inlineStr">
         <is>
@@ -10299,40 +10305,40 @@
         </is>
       </c>
       <c r="H132" s="20" t="n">
-        <v>134.466</v>
+        <v>4.842</v>
       </c>
       <c r="I132" s="20" t="n">
-        <v>2.916295653927599</v>
+        <v>2.0057023</v>
       </c>
       <c r="J132" s="22" t="n">
-        <v>34.35404370485792</v>
+        <v>-1.43550383550229</v>
       </c>
       <c r="K132" s="22" t="n">
-        <v>6.90904715732555</v>
+        <v>27.15453070970258</v>
       </c>
       <c r="L132" s="22" t="n">
-        <v>0.39782078028546</v>
+        <v>43.79434694279223</v>
       </c>
       <c r="M132" s="20" t="n">
-        <v>29.52748942714341</v>
+        <v>0.1557346455313411</v>
       </c>
       <c r="N132" s="22" t="n">
-        <v>6.521741571708831</v>
+        <v>46.96048918565198</v>
       </c>
       <c r="O132" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P132" s="20" t="n">
-        <v>0.9920879293908172</v>
+        <v>1</v>
       </c>
       <c r="Q132" s="15" t="inlineStr">
         <is>
-          <t>Reportable Segments Re (100%)</t>
+          <t>Single Reportable (100%)</t>
         </is>
       </c>
       <c r="R132" s="17" t="inlineStr">
         <is>
-          <t>Reportable Segments Retail 100%; Reportable Segments Credit 0%</t>
+          <t>Single Reportable 100%</t>
         </is>
       </c>
       <c r="S132" s="18" t="n">
@@ -10341,7 +10347,7 @@
       <c r="T132" s="17" t="n"/>
       <c r="U132" s="15" t="inlineStr">
         <is>
-          <t>Reportable Segments  +1%</t>
+          <t>Single Reportable +64%</t>
         </is>
       </c>
     </row>
@@ -10351,12 +10357,12 @@
       </c>
       <c r="B133" s="14" t="inlineStr">
         <is>
-          <t>AKBA</t>
+          <t>CATO</t>
         </is>
       </c>
       <c r="C133" s="15" t="inlineStr">
         <is>
-          <t>Akebia Therapeutics, Inc.</t>
+          <t>The Cato Corporation</t>
         </is>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -10366,11 +10372,11 @@
       </c>
       <c r="E133" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discr</t>
         </is>
       </c>
       <c r="F133" s="18" t="n">
-        <v>305814400</v>
+        <v>66662584</v>
       </c>
       <c r="G133" s="19" t="inlineStr">
         <is>
@@ -10378,42 +10384,40 @@
         </is>
       </c>
       <c r="H133" s="20" t="n">
-        <v>28.087</v>
-      </c>
-      <c r="I133" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>134.466</v>
+      </c>
+      <c r="I133" s="20" t="n">
+        <v>2.916295653927599</v>
       </c>
       <c r="J133" s="22" t="n">
-        <v>21.06320195668403</v>
+        <v>34.35404370485792</v>
       </c>
       <c r="K133" s="22" t="n">
-        <v>-20.3691903301605</v>
+        <v>6.90904715732555</v>
       </c>
       <c r="L133" s="22" t="n">
-        <v>9.19871632034412</v>
+        <v>0.39782078028546</v>
       </c>
       <c r="M133" s="20" t="n">
-        <v>-6.123532931375708</v>
+        <v>29.52748942714341</v>
       </c>
       <c r="N133" s="22" t="n">
-        <v>-58.26771816145106</v>
+        <v>6.521741571708831</v>
       </c>
       <c r="O133" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P133" s="20" t="n">
-        <v>1</v>
+        <v>0.9920879293908172</v>
       </c>
       <c r="Q133" s="15" t="inlineStr">
         <is>
-          <t>Reportable (100%)</t>
+          <t>Reportable Segments Re (100%)</t>
         </is>
       </c>
       <c r="R133" s="17" t="inlineStr">
         <is>
-          <t>Reportable 100%</t>
+          <t>Reportable Segments Retail 100%; Reportable Segments Credit 0%</t>
         </is>
       </c>
       <c r="S133" s="18" t="n">
@@ -10422,7 +10426,7 @@
       <c r="T133" s="17" t="n"/>
       <c r="U133" s="15" t="inlineStr">
         <is>
-          <t>Reportable -77%</t>
+          <t>Reportable Segments  +1%</t>
         </is>
       </c>
     </row>
@@ -10432,12 +10436,12 @@
       </c>
       <c r="B134" s="14" t="inlineStr">
         <is>
-          <t>SIRI</t>
+          <t>AKBA</t>
         </is>
       </c>
       <c r="C134" s="15" t="inlineStr">
         <is>
-          <t>Sirius XM Holdings Inc.</t>
+          <t>Akebia Therapeutics, Inc.</t>
         </is>
       </c>
       <c r="D134" s="16" t="inlineStr">
@@ -10447,11 +10451,11 @@
       </c>
       <c r="E134" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Communication </t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F134" s="18" t="n">
-        <v>9543175168</v>
+        <v>305814400</v>
       </c>
       <c r="G134" s="19" t="inlineStr">
         <is>
@@ -10459,40 +10463,42 @@
         </is>
       </c>
       <c r="H134" s="20" t="n">
-        <v>7.839</v>
-      </c>
-      <c r="I134" s="20" t="n">
-        <v>12.0127125</v>
+        <v>28.087</v>
+      </c>
+      <c r="I134" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J134" s="22" t="n">
-        <v>12.80212302889506</v>
+        <v>21.06320195668403</v>
       </c>
       <c r="K134" s="22" t="n">
-        <v>10.57658645741083</v>
+        <v>-20.3691903301605</v>
       </c>
       <c r="L134" s="22" t="n">
-        <v>25.19519869479081</v>
+        <v>9.19871632034412</v>
       </c>
       <c r="M134" s="20" t="n">
-        <v>4.4736355226642</v>
+        <v>-6.123532931375708</v>
       </c>
       <c r="N134" s="22" t="n">
-        <v>37.51723087267589</v>
+        <v>-58.26771816145106</v>
       </c>
       <c r="O134" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P134" s="20" t="n">
-        <v>0.6308860972502057</v>
+        <v>1</v>
       </c>
       <c r="Q134" s="15" t="inlineStr">
         <is>
-          <t>Sirius XM (76%)</t>
+          <t>Reportable (100%)</t>
         </is>
       </c>
       <c r="R134" s="17" t="inlineStr">
         <is>
-          <t>Sirius XM 76%; Pandora And Off Platform 24%</t>
+          <t>Reportable 100%</t>
         </is>
       </c>
       <c r="S134" s="18" t="n">
@@ -10501,7 +10507,7 @@
       <c r="T134" s="17" t="n"/>
       <c r="U134" s="15" t="inlineStr">
         <is>
-          <t>Pandora And Off Plat -0%</t>
+          <t>Reportable -77%</t>
         </is>
       </c>
     </row>
@@ -10511,12 +10517,12 @@
       </c>
       <c r="B135" s="14" t="inlineStr">
         <is>
-          <t>HURC</t>
+          <t>SIRI</t>
         </is>
       </c>
       <c r="C135" s="15" t="inlineStr">
         <is>
-          <t>Hurco Companies, Inc.</t>
+          <t>Sirius XM Holdings Inc.</t>
         </is>
       </c>
       <c r="D135" s="16" t="inlineStr">
@@ -10526,11 +10532,11 @@
       </c>
       <c r="E135" s="17" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t xml:space="preserve">Communication </t>
         </is>
       </c>
       <c r="F135" s="18" t="n">
-        <v>145911536</v>
+        <v>9543175168</v>
       </c>
       <c r="G135" s="19" t="inlineStr">
         <is>
@@ -10538,47 +10544,51 @@
         </is>
       </c>
       <c r="H135" s="20" t="n">
-        <v>-6.862805819592628</v>
-      </c>
-      <c r="I135" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>7.839</v>
+      </c>
+      <c r="I135" s="20" t="n">
+        <v>12.0127125</v>
       </c>
       <c r="J135" s="22" t="n">
-        <v>3.75916957537465</v>
+        <v>12.80212302889506</v>
       </c>
       <c r="K135" s="22" t="n">
-        <v>-6.10196397965777</v>
+        <v>10.57658645741083</v>
       </c>
       <c r="L135" s="22" t="n">
-        <v>-5.89115926129091</v>
+        <v>25.19519869479081</v>
       </c>
       <c r="M135" s="20" t="n">
-        <v>3.535305528612997</v>
+        <v>4.4736355226642</v>
       </c>
       <c r="N135" s="22" t="n">
-        <v>11.83590644756314</v>
+        <v>37.51723087267589</v>
       </c>
       <c r="O135" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P135" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q135" s="15" t="n"/>
-      <c r="R135" s="17" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="P135" s="20" t="n">
+        <v>0.6308860972502057</v>
+      </c>
+      <c r="Q135" s="15" t="inlineStr">
+        <is>
+          <t>Sirius XM (76%)</t>
+        </is>
+      </c>
+      <c r="R135" s="17" t="inlineStr">
+        <is>
+          <t>Sirius XM 76%; Pandora And Off Platform 24%</t>
+        </is>
+      </c>
       <c r="S135" s="18" t="n">
-        <v>9</v>
-      </c>
-      <c r="T135" s="17" t="inlineStr">
-        <is>
-          <t>Europe 26%; Americas 21%; US 20%</t>
-        </is>
-      </c>
-      <c r="U135" s="15" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="T135" s="17" t="n"/>
+      <c r="U135" s="15" t="inlineStr">
+        <is>
+          <t>Pandora And Off Plat -0%</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="13" t="n">
@@ -10586,12 +10596,12 @@
       </c>
       <c r="B136" s="14" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>HURC</t>
         </is>
       </c>
       <c r="C136" s="15" t="inlineStr">
         <is>
-          <t>Coffee Holding Co., Inc.</t>
+          <t>Hurco Companies, Inc.</t>
         </is>
       </c>
       <c r="D136" s="16" t="inlineStr">
@@ -10601,11 +10611,11 @@
       </c>
       <c r="E136" s="17" t="inlineStr">
         <is>
-          <t>Consumer Stapl</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F136" s="18" t="n">
-        <v>19123810</v>
+        <v>145911536</v>
       </c>
       <c r="G136" s="19" t="inlineStr">
         <is>
@@ -10613,51 +10623,47 @@
         </is>
       </c>
       <c r="H136" s="20" t="n">
-        <v>6.732</v>
-      </c>
-      <c r="I136" s="20" t="n">
-        <v>12.407407</v>
+        <v>-6.862805819592628</v>
+      </c>
+      <c r="I136" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J136" s="22" t="n">
-        <v>42.03289398842584</v>
+        <v>3.75916957537465</v>
       </c>
       <c r="K136" s="22" t="n">
-        <v>14.9836891396905</v>
+        <v>-6.10196397965777</v>
       </c>
       <c r="L136" s="22" t="n">
-        <v>4.4448932469455</v>
+        <v>-5.89115926129091</v>
       </c>
       <c r="M136" s="20" t="n">
-        <v>0.4654342573568866</v>
+        <v>3.535305528612997</v>
       </c>
       <c r="N136" s="22" t="n">
-        <v>25.28308922858965</v>
+        <v>11.83590644756314</v>
       </c>
       <c r="O136" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P136" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q136" s="15" t="inlineStr">
-        <is>
-          <t>Operating (100%)</t>
-        </is>
-      </c>
-      <c r="R136" s="17" t="inlineStr">
-        <is>
-          <t>Operating 100%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P136" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q136" s="15" t="n"/>
+      <c r="R136" s="17" t="n"/>
       <c r="S136" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T136" s="17" t="n"/>
-      <c r="U136" s="15" t="inlineStr">
-        <is>
-          <t>Operating +23%</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="T136" s="17" t="inlineStr">
+        <is>
+          <t>Europe 26%; Americas 21%; US 20%</t>
+        </is>
+      </c>
+      <c r="U136" s="15" t="n"/>
     </row>
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="13" t="n">
@@ -10665,12 +10671,12 @@
       </c>
       <c r="B137" s="14" t="inlineStr">
         <is>
-          <t>CLFD</t>
+          <t>JVA</t>
         </is>
       </c>
       <c r="C137" s="15" t="inlineStr">
         <is>
-          <t>Clearfield, Inc.</t>
+          <t>Coffee Holding Co., Inc.</t>
         </is>
       </c>
       <c r="D137" s="16" t="inlineStr">
@@ -10680,11 +10686,11 @@
       </c>
       <c r="E137" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t>Consumer Stapl</t>
         </is>
       </c>
       <c r="F137" s="18" t="n">
-        <v>524960864</v>
+        <v>19123810</v>
       </c>
       <c r="G137" s="19" t="inlineStr">
         <is>
@@ -10692,45 +10698,51 @@
         </is>
       </c>
       <c r="H137" s="20" t="n">
-        <v>91.926</v>
+        <v>6.732</v>
       </c>
       <c r="I137" s="20" t="n">
-        <v>167.95653</v>
+        <v>12.407407</v>
       </c>
       <c r="J137" s="22" t="n">
-        <v>2.22637049013564</v>
+        <v>42.03289398842584</v>
       </c>
       <c r="K137" s="22" t="n">
-        <v>-0.9055781066418901</v>
+        <v>14.9836891396905</v>
       </c>
       <c r="L137" s="22" t="n">
-        <v>10.26651185578426</v>
+        <v>4.4448932469455</v>
       </c>
       <c r="M137" s="20" t="n">
-        <v>-5.776034516571877</v>
+        <v>0.4654342573568866</v>
       </c>
       <c r="N137" s="22" t="n">
-        <v>11.62432290838696</v>
+        <v>25.28308922858965</v>
       </c>
       <c r="O137" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P137" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="Q137" s="15" t="n"/>
-      <c r="R137" s="17" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="P137" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q137" s="15" t="inlineStr">
+        <is>
+          <t>Operating (100%)</t>
+        </is>
+      </c>
+      <c r="R137" s="17" t="inlineStr">
+        <is>
+          <t>Operating 100%</t>
+        </is>
+      </c>
       <c r="S137" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="T137" s="17" t="inlineStr">
-        <is>
-          <t>US 97%; Non Us 3%</t>
-        </is>
-      </c>
-      <c r="U137" s="15" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="T137" s="17" t="n"/>
+      <c r="U137" s="15" t="inlineStr">
+        <is>
+          <t>Operating +23%</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="13" t="n">
@@ -10738,12 +10750,12 @@
       </c>
       <c r="B138" s="14" t="inlineStr">
         <is>
-          <t>PROV</t>
+          <t>CLFD</t>
         </is>
       </c>
       <c r="C138" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provident Financial Holdings, </t>
+          <t>Clearfield, Inc.</t>
         </is>
       </c>
       <c r="D138" s="16" t="inlineStr">
@@ -10753,43 +10765,37 @@
       </c>
       <c r="E138" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F138" s="18" t="n">
-        <v>107563488</v>
+        <v>524960864</v>
       </c>
       <c r="G138" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H138" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H138" s="20" t="n">
+        <v>91.926</v>
       </c>
       <c r="I138" s="20" t="n">
-        <v>18.494625</v>
+        <v>167.95653</v>
       </c>
       <c r="J138" s="22" t="n">
-        <v>8.407967835537141</v>
-      </c>
-      <c r="K138" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>2.22637049013564</v>
+      </c>
+      <c r="K138" s="22" t="n">
+        <v>-0.9055781066418901</v>
       </c>
       <c r="L138" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M138" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>10.26651185578426</v>
+      </c>
+      <c r="M138" s="20" t="n">
+        <v>-5.776034516571877</v>
       </c>
       <c r="N138" s="22" t="n">
-        <v>13.3670912336621</v>
+        <v>11.62432290838696</v>
       </c>
       <c r="O138" s="18" t="n">
         <v>0</v>
@@ -10802,9 +10808,13 @@
       <c r="Q138" s="15" t="n"/>
       <c r="R138" s="17" t="n"/>
       <c r="S138" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T138" s="17" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="T138" s="17" t="inlineStr">
+        <is>
+          <t>US 97%; Non Us 3%</t>
+        </is>
+      </c>
       <c r="U138" s="15" t="n"/>
     </row>
     <row r="139" ht="16" customHeight="1">
@@ -10813,12 +10823,12 @@
       </c>
       <c r="B139" s="14" t="inlineStr">
         <is>
-          <t>CODA</t>
+          <t>PROV</t>
         </is>
       </c>
       <c r="C139" s="15" t="inlineStr">
         <is>
-          <t>Coda Octopus Group, Inc.</t>
+          <t xml:space="preserve">Provident Financial Holdings, </t>
         </is>
       </c>
       <c r="D139" s="16" t="inlineStr">
@@ -10828,67 +10838,59 @@
       </c>
       <c r="E139" s="17" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F139" s="18" t="n">
-        <v>108295240</v>
+        <v>107563488</v>
       </c>
       <c r="G139" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H139" s="20" t="n">
-        <v>11.138</v>
+      <c r="H139" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="I139" s="20" t="n">
-        <v>21.333334</v>
+        <v>18.494625</v>
       </c>
       <c r="J139" s="22" t="n">
-        <v>1.84264170445135</v>
-      </c>
-      <c r="K139" s="22" t="n">
-        <v>16.80549850408138</v>
+        <v>8.407967835537141</v>
+      </c>
+      <c r="K139" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L139" s="22" t="n">
-        <v>24.49495025980879</v>
-      </c>
-      <c r="M139" s="20" t="n">
-        <v>-4.37058436058821</v>
+        <v>0</v>
+      </c>
+      <c r="M139" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N139" s="22" t="n">
-        <v>63.28571864536831</v>
+        <v>13.3670912336621</v>
       </c>
       <c r="O139" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="P139" s="20" t="n">
-        <v>0.425811579408509</v>
-      </c>
-      <c r="Q139" s="15" t="inlineStr">
-        <is>
-          <t>Marine Technology Busi (56%)</t>
-        </is>
-      </c>
-      <c r="R139" s="17" t="inlineStr">
-        <is>
-          <t>Marine Technology Business Products 56%; Defense Engineering Services Business S</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P139" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="Q139" s="15" t="n"/>
+      <c r="R139" s="17" t="n"/>
       <c r="S139" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="T139" s="17" t="inlineStr">
-        <is>
-          <t>Americas 35%; Europe 31%; Australia And Asia 28%</t>
-        </is>
-      </c>
-      <c r="U139" s="15" t="inlineStr">
-        <is>
-          <t>Defense Engineering  +6%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T139" s="17" t="n"/>
+      <c r="U139" s="15" t="n"/>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="13" t="n">
@@ -10896,12 +10898,12 @@
       </c>
       <c r="B140" s="14" t="inlineStr">
         <is>
-          <t>SIEB</t>
+          <t>CODA</t>
         </is>
       </c>
       <c r="C140" s="15" t="inlineStr">
         <is>
-          <t>Siebert Financial Corp.</t>
+          <t>Coda Octopus Group, Inc.</t>
         </is>
       </c>
       <c r="D140" s="16" t="inlineStr">
@@ -10911,67 +10913,65 @@
       </c>
       <c r="E140" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="F140" s="18" t="n">
-        <v>69599592</v>
+        <v>108295240</v>
       </c>
       <c r="G140" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H140" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I140" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J140" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H140" s="20" t="n">
+        <v>11.138</v>
+      </c>
+      <c r="I140" s="20" t="n">
+        <v>21.333334</v>
+      </c>
+      <c r="J140" s="22" t="n">
+        <v>1.84264170445135</v>
       </c>
       <c r="K140" s="22" t="n">
-        <v>5.17888936540735</v>
+        <v>16.80549850408138</v>
       </c>
       <c r="L140" s="22" t="n">
-        <v>7.23199371130981</v>
+        <v>24.49495025980879</v>
       </c>
       <c r="M140" s="20" t="n">
-        <v>-1.897588315217392</v>
+        <v>-4.37058436058821</v>
       </c>
       <c r="N140" s="22" t="n">
-        <v>-64.87603317998357</v>
+        <v>63.28571864536831</v>
       </c>
       <c r="O140" s="18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P140" s="20" t="n">
-        <v>0.9865046689171856</v>
+        <v>0.425811579408509</v>
       </c>
       <c r="Q140" s="15" t="inlineStr">
         <is>
-          <t>Financial Services (99%)</t>
+          <t>Marine Technology Busi (56%)</t>
         </is>
       </c>
       <c r="R140" s="17" t="inlineStr">
         <is>
-          <t>Financial Services 99%; Media Sports And Entertainment 1%</t>
+          <t>Marine Technology Business Products 56%; Defense Engineering Services Business S</t>
         </is>
       </c>
       <c r="S140" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T140" s="17" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="T140" s="17" t="inlineStr">
+        <is>
+          <t>Americas 35%; Europe 31%; Australia And Asia 28%</t>
+        </is>
+      </c>
       <c r="U140" s="15" t="inlineStr">
         <is>
-          <t>Financial Services +11%</t>
+          <t>Defense Engineering  +6%</t>
         </is>
       </c>
     </row>
@@ -16759,12 +16759,12 @@
       </c>
       <c r="B215" s="14" t="inlineStr">
         <is>
-          <t>ALGM</t>
+          <t>ETST</t>
         </is>
       </c>
       <c r="C215" s="15" t="inlineStr">
         <is>
-          <t>Allegro MicroSystems, Inc.</t>
+          <t>Earth Science Tech, Inc.</t>
         </is>
       </c>
       <c r="D215" s="16" t="inlineStr">
@@ -16774,39 +16774,39 @@
       </c>
       <c r="E215" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F215" s="18" t="n">
-        <v>10785431552</v>
-      </c>
-      <c r="G215" s="24" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+        <v>43226132</v>
+      </c>
+      <c r="G215" s="19" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="H215" s="20" t="n">
-        <v>102.984</v>
-      </c>
-      <c r="I215" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J215" s="22" t="n">
-        <v>1.45955566109384</v>
+        <v>9.584</v>
+      </c>
+      <c r="I215" s="20" t="n">
+        <v>15.000001</v>
+      </c>
+      <c r="J215" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="K215" s="22" t="n">
-        <v>1.72249294213012</v>
+        <v>53.80440161697887</v>
       </c>
       <c r="L215" s="22" t="n">
-        <v>8.40662130826337</v>
+        <v>10.49770988671045</v>
       </c>
       <c r="M215" s="20" t="n">
-        <v>1.583960335173133</v>
+        <v>-0.1533199794407697</v>
       </c>
       <c r="N215" s="22" t="n">
-        <v>77.3446585625084</v>
+        <v>-15.78947450975963</v>
       </c>
       <c r="O215" s="18" t="n">
         <v>0</v>
@@ -16819,13 +16819,9 @@
       <c r="Q215" s="15" t="n"/>
       <c r="R215" s="17" t="n"/>
       <c r="S215" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="T215" s="17" t="inlineStr">
-        <is>
-          <t>CN 27%; JP 19%; Europe 15%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T215" s="17" t="n"/>
       <c r="U215" s="15" t="n"/>
     </row>
     <row r="216" ht="16" customHeight="1">
@@ -16834,12 +16830,12 @@
       </c>
       <c r="B216" s="14" t="inlineStr">
         <is>
-          <t>SFST</t>
+          <t>ALGM</t>
         </is>
       </c>
       <c r="C216" s="15" t="inlineStr">
         <is>
-          <t>Southern First Bancshares, Inc</t>
+          <t>Allegro MicroSystems, Inc.</t>
         </is>
       </c>
       <c r="D216" s="16" t="inlineStr">
@@ -16849,43 +16845,39 @@
       </c>
       <c r="E216" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F216" s="18" t="n">
-        <v>578939776</v>
-      </c>
-      <c r="G216" s="19" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
-        </is>
-      </c>
-      <c r="H216" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I216" s="20" t="n">
-        <v>14.373239</v>
+        <v>10785431552</v>
+      </c>
+      <c r="G216" s="24" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="H216" s="20" t="n">
+        <v>102.984</v>
+      </c>
+      <c r="I216" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J216" s="22" t="n">
-        <v>3.03631449834383</v>
-      </c>
-      <c r="K216" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>1.45955566109384</v>
+      </c>
+      <c r="K216" s="22" t="n">
+        <v>1.72249294213012</v>
       </c>
       <c r="L216" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M216" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>8.40662130826337</v>
+      </c>
+      <c r="M216" s="20" t="n">
+        <v>1.583960335173133</v>
       </c>
       <c r="N216" s="22" t="n">
-        <v>46.83578253190569</v>
+        <v>77.3446585625084</v>
       </c>
       <c r="O216" s="18" t="n">
         <v>0</v>
@@ -16898,9 +16890,13 @@
       <c r="Q216" s="15" t="n"/>
       <c r="R216" s="17" t="n"/>
       <c r="S216" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T216" s="17" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="T216" s="17" t="inlineStr">
+        <is>
+          <t>CN 27%; JP 19%; Europe 15%</t>
+        </is>
+      </c>
       <c r="U216" s="15" t="n"/>
     </row>
     <row r="217" ht="16" customHeight="1">
@@ -16909,12 +16905,12 @@
       </c>
       <c r="B217" s="14" t="inlineStr">
         <is>
-          <t>FATN</t>
+          <t>SFST</t>
         </is>
       </c>
       <c r="C217" s="15" t="inlineStr">
         <is>
-          <t>FatPipe Inc. Common Stock</t>
+          <t>Southern First Bancshares, Inc</t>
         </is>
       </c>
       <c r="D217" s="16" t="inlineStr">
@@ -16924,37 +16920,43 @@
       </c>
       <c r="E217" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F217" s="18" t="n">
-        <v>84707784</v>
+        <v>578939776</v>
       </c>
       <c r="G217" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H217" s="20" t="n">
-        <v>21.523</v>
+      <c r="H217" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="I217" s="20" t="n">
-        <v>17.257143</v>
+        <v>14.373239</v>
       </c>
       <c r="J217" s="22" t="n">
-        <v>-1.45887439123651</v>
-      </c>
-      <c r="K217" s="22" t="n">
-        <v>14.34799023925575</v>
+        <v>3.03631449834383</v>
+      </c>
+      <c r="K217" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L217" s="22" t="n">
-        <v>14.43825219466334</v>
-      </c>
-      <c r="M217" s="20" t="n">
-        <v>-0.1617276693742073</v>
+        <v>0</v>
+      </c>
+      <c r="M217" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N217" s="22" t="n">
-        <v>-55.9613349104299</v>
+        <v>46.83578253190569</v>
       </c>
       <c r="O217" s="18" t="n">
         <v>0</v>
@@ -16967,13 +16969,9 @@
       <c r="Q217" s="15" t="n"/>
       <c r="R217" s="17" t="n"/>
       <c r="S217" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="T217" s="17" t="inlineStr">
-        <is>
-          <t>US 96%; Non Us 4%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T217" s="17" t="n"/>
       <c r="U217" s="15" t="n"/>
     </row>
     <row r="218" ht="16" customHeight="1">
@@ -16982,12 +16980,12 @@
       </c>
       <c r="B218" s="14" t="inlineStr">
         <is>
-          <t>ALNY</t>
+          <t>FATN</t>
         </is>
       </c>
       <c r="C218" s="15" t="inlineStr">
         <is>
-          <t>Alnylam Pharmaceuticals, Inc.</t>
+          <t>FatPipe Inc. Common Stock</t>
         </is>
       </c>
       <c r="D218" s="16" t="inlineStr">
@@ -16997,11 +16995,11 @@
       </c>
       <c r="E218" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F218" s="18" t="n">
-        <v>38901559296</v>
+        <v>84707784</v>
       </c>
       <c r="G218" s="19" t="inlineStr">
         <is>
@@ -17009,25 +17007,25 @@
         </is>
       </c>
       <c r="H218" s="20" t="n">
-        <v>48.16</v>
+        <v>21.523</v>
       </c>
       <c r="I218" s="20" t="n">
-        <v>73.02506</v>
+        <v>17.257143</v>
       </c>
       <c r="J218" s="22" t="n">
-        <v>1.61995031088219</v>
+        <v>-1.45887439123651</v>
       </c>
       <c r="K218" s="22" t="n">
-        <v>-131.6113410564707</v>
+        <v>14.34799023925575</v>
       </c>
       <c r="L218" s="22" t="n">
-        <v>21.56497795738342</v>
+        <v>14.43825219466334</v>
       </c>
       <c r="M218" s="20" t="n">
-        <v>-1.878003059036814</v>
+        <v>-0.1617276693742073</v>
       </c>
       <c r="N218" s="22" t="n">
-        <v>2.92387965641219</v>
+        <v>-55.9613349104299</v>
       </c>
       <c r="O218" s="18" t="n">
         <v>0</v>
@@ -17040,11 +17038,11 @@
       <c r="Q218" s="15" t="n"/>
       <c r="R218" s="17" t="n"/>
       <c r="S218" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T218" s="17" t="inlineStr">
         <is>
-          <t>US 64%; Europe 26%; Non US Or Europe 10%</t>
+          <t>US 96%; Non Us 4%</t>
         </is>
       </c>
       <c r="U218" s="15" t="n"/>
@@ -17055,12 +17053,12 @@
       </c>
       <c r="B219" s="14" t="inlineStr">
         <is>
-          <t>LC</t>
+          <t>ALNY</t>
         </is>
       </c>
       <c r="C219" s="15" t="inlineStr">
         <is>
-          <t>LendingClub Corporation</t>
+          <t>Alnylam Pharmaceuticals, Inc.</t>
         </is>
       </c>
       <c r="D219" s="16" t="inlineStr">
@@ -17070,11 +17068,11 @@
       </c>
       <c r="E219" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F219" s="18" t="n">
-        <v>2215891200</v>
+        <v>38901559296</v>
       </c>
       <c r="G219" s="19" t="inlineStr">
         <is>
@@ -17082,29 +17080,25 @@
         </is>
       </c>
       <c r="H219" s="20" t="n">
-        <v>4.862</v>
+        <v>48.16</v>
       </c>
       <c r="I219" s="20" t="n">
-        <v>12.806666</v>
+        <v>73.02506</v>
       </c>
       <c r="J219" s="22" t="n">
-        <v>-97.55883274375822</v>
-      </c>
-      <c r="K219" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>1.61995031088219</v>
+      </c>
+      <c r="K219" s="22" t="n">
+        <v>-131.6113410564707</v>
       </c>
       <c r="L219" s="22" t="n">
-        <v>21.381001</v>
-      </c>
-      <c r="M219" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>21.56497795738342</v>
+      </c>
+      <c r="M219" s="20" t="n">
+        <v>-1.878003059036814</v>
       </c>
       <c r="N219" s="22" t="n">
-        <v>47.2143524830653</v>
+        <v>2.92387965641219</v>
       </c>
       <c r="O219" s="18" t="n">
         <v>0</v>
@@ -17117,9 +17111,13 @@
       <c r="Q219" s="15" t="n"/>
       <c r="R219" s="17" t="n"/>
       <c r="S219" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T219" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="T219" s="17" t="inlineStr">
+        <is>
+          <t>US 64%; Europe 26%; Non US Or Europe 10%</t>
+        </is>
+      </c>
       <c r="U219" s="15" t="n"/>
     </row>
     <row r="220" ht="16" customHeight="1">
@@ -17128,12 +17126,12 @@
       </c>
       <c r="B220" s="14" t="inlineStr">
         <is>
-          <t>ASAN</t>
+          <t>LC</t>
         </is>
       </c>
       <c r="C220" s="15" t="inlineStr">
         <is>
-          <t>Asana, Inc.</t>
+          <t>LendingClub Corporation</t>
         </is>
       </c>
       <c r="D220" s="16" t="inlineStr">
@@ -17143,11 +17141,11 @@
       </c>
       <c r="E220" s="17" t="inlineStr">
         <is>
-          <t>Information Te</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F220" s="18" t="n">
-        <v>1606653440</v>
+        <v>2215891200</v>
       </c>
       <c r="G220" s="19" t="inlineStr">
         <is>
@@ -17155,27 +17153,29 @@
         </is>
       </c>
       <c r="H220" s="20" t="n">
-        <v>-8.123680517291266</v>
-      </c>
-      <c r="I220" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>4.862</v>
+      </c>
+      <c r="I220" s="20" t="n">
+        <v>12.806666</v>
       </c>
       <c r="J220" s="22" t="n">
-        <v>5.21506708496677</v>
-      </c>
-      <c r="K220" s="22" t="n">
-        <v>593.3103900360537</v>
+        <v>-97.55883274375822</v>
+      </c>
+      <c r="K220" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L220" s="22" t="n">
-        <v>-20.10379283920456</v>
-      </c>
-      <c r="M220" s="20" t="n">
-        <v>1.161307569410374</v>
+        <v>21.381001</v>
+      </c>
+      <c r="M220" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N220" s="22" t="n">
-        <v>-65.68898774779171</v>
+        <v>47.2143524830653</v>
       </c>
       <c r="O220" s="18" t="n">
         <v>0</v>
@@ -17188,13 +17188,9 @@
       <c r="Q220" s="15" t="n"/>
       <c r="R220" s="17" t="n"/>
       <c r="S220" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="T220" s="17" t="inlineStr">
-        <is>
-          <t>US 60%; Non Us 40%</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T220" s="17" t="n"/>
       <c r="U220" s="15" t="n"/>
     </row>
     <row r="221" ht="16" customHeight="1">
@@ -17203,12 +17199,12 @@
       </c>
       <c r="B221" s="14" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>ASAN</t>
         </is>
       </c>
       <c r="C221" s="15" t="inlineStr">
         <is>
-          <t>Instil Bio, Inc.</t>
+          <t>Asana, Inc.</t>
         </is>
       </c>
       <c r="D221" s="16" t="inlineStr">
@@ -17218,11 +17214,11 @@
       </c>
       <c r="E221" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Te</t>
         </is>
       </c>
       <c r="F221" s="18" t="n">
-        <v>50390088</v>
+        <v>1606653440</v>
       </c>
       <c r="G221" s="19" t="inlineStr">
         <is>
@@ -17230,7 +17226,7 @@
         </is>
       </c>
       <c r="H221" s="20" t="n">
-        <v>-0.908630976186148</v>
+        <v>-8.123680517291266</v>
       </c>
       <c r="I221" s="21" t="inlineStr">
         <is>
@@ -17238,19 +17234,19 @@
         </is>
       </c>
       <c r="J221" s="22" t="n">
-        <v>-99.73588426442328</v>
+        <v>5.21506708496677</v>
       </c>
       <c r="K221" s="22" t="n">
-        <v>-71.9501116620614</v>
+        <v>593.3103900360537</v>
       </c>
       <c r="L221" s="22" t="n">
-        <v>0</v>
+        <v>-20.10379283920456</v>
       </c>
       <c r="M221" s="20" t="n">
-        <v>-1.184148336666061</v>
+        <v>1.161307569410374</v>
       </c>
       <c r="N221" s="22" t="n">
-        <v>-45.50979428646714</v>
+        <v>-65.68898774779171</v>
       </c>
       <c r="O221" s="18" t="n">
         <v>0</v>
@@ -17263,9 +17259,13 @@
       <c r="Q221" s="15" t="n"/>
       <c r="R221" s="17" t="n"/>
       <c r="S221" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T221" s="17" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="T221" s="17" t="inlineStr">
+        <is>
+          <t>US 60%; Non Us 40%</t>
+        </is>
+      </c>
       <c r="U221" s="15" t="n"/>
     </row>
     <row r="222" ht="16" customHeight="1">
@@ -17274,12 +17274,12 @@
       </c>
       <c r="B222" s="14" t="inlineStr">
         <is>
-          <t>CBKM</t>
+          <t>TIL</t>
         </is>
       </c>
       <c r="C222" s="15" t="inlineStr">
         <is>
-          <t>Consumers Bancorp, Inc.</t>
+          <t>Instil Bio, Inc.</t>
         </is>
       </c>
       <c r="D222" s="16" t="inlineStr">
@@ -17289,43 +17289,39 @@
       </c>
       <c r="E222" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="F222" s="18" t="n">
-        <v>92739416</v>
+        <v>50390088</v>
       </c>
       <c r="G222" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H222" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I222" s="20" t="n">
-        <v>8.829342</v>
+      <c r="H222" s="20" t="n">
+        <v>-0.908630976186148</v>
+      </c>
+      <c r="I222" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="J222" s="22" t="n">
-        <v>11.2038687095359</v>
-      </c>
-      <c r="K222" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>-99.73588426442328</v>
+      </c>
+      <c r="K222" s="22" t="n">
+        <v>-71.9501116620614</v>
       </c>
       <c r="L222" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="M222" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="M222" s="20" t="n">
+        <v>-1.184148336666061</v>
       </c>
       <c r="N222" s="22" t="n">
-        <v>44.15947036183197</v>
+        <v>-45.50979428646714</v>
       </c>
       <c r="O222" s="18" t="n">
         <v>0</v>
@@ -17349,12 +17345,12 @@
       </c>
       <c r="B223" s="14" t="inlineStr">
         <is>
-          <t>ETST</t>
+          <t>CBKM</t>
         </is>
       </c>
       <c r="C223" s="15" t="inlineStr">
         <is>
-          <t>Earth Science Tech, Inc.</t>
+          <t>Consumers Bancorp, Inc.</t>
         </is>
       </c>
       <c r="D223" s="16" t="inlineStr">
@@ -17364,39 +17360,43 @@
       </c>
       <c r="E223" s="17" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F223" s="18" t="n">
-        <v>43226132</v>
+        <v>92739416</v>
       </c>
       <c r="G223" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H223" s="20" t="n">
-        <v>9.584</v>
+      <c r="H223" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="I223" s="20" t="n">
-        <v>15.000001</v>
-      </c>
-      <c r="J223" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K223" s="22" t="n">
-        <v>53.80440161697887</v>
+        <v>8.829342</v>
+      </c>
+      <c r="J223" s="22" t="n">
+        <v>11.2038687095359</v>
+      </c>
+      <c r="K223" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L223" s="22" t="n">
-        <v>10.49770988671045</v>
-      </c>
-      <c r="M223" s="20" t="n">
-        <v>-0.1533199794407697</v>
+        <v>0</v>
+      </c>
+      <c r="M223" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N223" s="22" t="n">
-        <v>-15.78947450975963</v>
+        <v>44.15947036183197</v>
       </c>
       <c r="O223" s="18" t="n">
         <v>0</v>
@@ -31079,12 +31079,12 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>WSFS</t>
+          <t>SIEB</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>WSFS Financial Corporation</t>
+          <t>Siebert Financial Corp.</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -31098,7 +31098,7 @@
         </is>
       </c>
       <c r="F29" s="18" t="n">
-        <v>4026127616</v>
+        <v>69599592</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
@@ -31110,42 +31110,42 @@
           <t>–</t>
         </is>
       </c>
-      <c r="I29" s="20" t="n">
-        <v>13.789661</v>
-      </c>
-      <c r="J29" s="22" t="n">
-        <v>6.158366732153779</v>
-      </c>
-      <c r="K29" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="I29" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J29" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K29" s="22" t="n">
+        <v>5.17888936540735</v>
       </c>
       <c r="L29" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>7.23199371130981</v>
+      </c>
+      <c r="M29" s="20" t="n">
+        <v>-1.897588315217392</v>
       </c>
       <c r="N29" s="22" t="n">
-        <v>37.01048893948796</v>
+        <v>-64.87603317998357</v>
       </c>
       <c r="O29" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P29" s="20" t="n">
-        <v>0.5461404223281471</v>
+        <v>0.9865046689171856</v>
       </c>
       <c r="Q29" s="15" t="inlineStr">
         <is>
-          <t>Wsfs Bank (70%)</t>
+          <t>Financial Services (99%)</t>
         </is>
       </c>
       <c r="R29" s="17" t="inlineStr">
         <is>
-          <t>Wsfs Bank 70%; Wealth Management 22%; Cash Connect 8%</t>
+          <t>Financial Services 99%; Media Sports And Entertainment 1%</t>
         </is>
       </c>
       <c r="S29" s="18" t="n">
@@ -31154,7 +31154,7 @@
       <c r="T29" s="17" t="n"/>
       <c r="U29" s="15" t="inlineStr">
         <is>
-          <t>Wealth Management +15%</t>
+          <t>Financial Services +11%</t>
         </is>
       </c>
     </row>
@@ -31164,12 +31164,12 @@
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>NRIM</t>
+          <t>WSFS</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>Northrim BanCorp, Inc.</t>
+          <t>WSFS Financial Corporation</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
@@ -31183,7 +31183,7 @@
         </is>
       </c>
       <c r="F30" s="18" t="n">
-        <v>621963648</v>
+        <v>4026127616</v>
       </c>
       <c r="G30" s="19" t="inlineStr">
         <is>
@@ -31196,10 +31196,10 @@
         </is>
       </c>
       <c r="I30" s="20" t="n">
-        <v>9.708333</v>
+        <v>13.789661</v>
       </c>
       <c r="J30" s="22" t="n">
-        <v>7.154905282262169</v>
+        <v>6.158366732153779</v>
       </c>
       <c r="K30" s="21" t="inlineStr">
         <is>
@@ -31215,22 +31215,22 @@
         </is>
       </c>
       <c r="N30" s="22" t="n">
-        <v>7.62249350229726</v>
+        <v>37.01048893948796</v>
       </c>
       <c r="O30" s="18" t="n">
         <v>3</v>
       </c>
       <c r="P30" s="20" t="n">
-        <v>0.6090673877493771</v>
+        <v>0.5461404223281471</v>
       </c>
       <c r="Q30" s="15" t="inlineStr">
         <is>
-          <t>Community Banking (76%)</t>
+          <t>Wsfs Bank (70%)</t>
         </is>
       </c>
       <c r="R30" s="17" t="inlineStr">
         <is>
-          <t>Community Banking 76%; Home Mortgage Lending 17%; Specialty Finance 7%</t>
+          <t>Wsfs Bank 70%; Wealth Management 22%; Cash Connect 8%</t>
         </is>
       </c>
       <c r="S30" s="18" t="n">
@@ -31239,7 +31239,7 @@
       <c r="T30" s="17" t="n"/>
       <c r="U30" s="15" t="inlineStr">
         <is>
-          <t>Specialty Finance +257%</t>
+          <t>Wealth Management +15%</t>
         </is>
       </c>
     </row>
@@ -31249,12 +31249,12 @@
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>CATO</t>
+          <t>NRIM</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>The Cato Corporation</t>
+          <t>Northrim BanCorp, Inc.</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -31264,52 +31264,58 @@
       </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
-          <t>Consumer Discr</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="F31" s="18" t="n">
-        <v>66662584</v>
+        <v>621963648</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H31" s="20" t="n">
-        <v>134.466</v>
+      <c r="H31" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="I31" s="20" t="n">
-        <v>2.916295653927599</v>
+        <v>9.708333</v>
       </c>
       <c r="J31" s="22" t="n">
-        <v>34.35404370485792</v>
-      </c>
-      <c r="K31" s="22" t="n">
-        <v>6.90904715732555</v>
+        <v>7.154905282262169</v>
+      </c>
+      <c r="K31" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="L31" s="22" t="n">
-        <v>0.39782078028546</v>
-      </c>
-      <c r="M31" s="20" t="n">
-        <v>29.52748942714341</v>
+        <v>0</v>
+      </c>
+      <c r="M31" s="21" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N31" s="22" t="n">
-        <v>6.521741571708831</v>
+        <v>7.62249350229726</v>
       </c>
       <c r="O31" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P31" s="20" t="n">
-        <v>0.9920879293908172</v>
+        <v>0.6090673877493771</v>
       </c>
       <c r="Q31" s="15" t="inlineStr">
         <is>
-          <t>Reportable Segments Re (100%)</t>
+          <t>Community Banking (76%)</t>
         </is>
       </c>
       <c r="R31" s="17" t="inlineStr">
         <is>
-          <t>Reportable Segments Retail 100%; Reportable Segments Credit 0%</t>
+          <t>Community Banking 76%; Home Mortgage Lending 17%; Specialty Finance 7%</t>
         </is>
       </c>
       <c r="S31" s="18" t="n">
@@ -31318,7 +31324,7 @@
       <c r="T31" s="17" t="n"/>
       <c r="U31" s="15" t="inlineStr">
         <is>
-          <t>Reportable Segments  +1%</t>
+          <t>Specialty Finance +257%</t>
         </is>
       </c>
     </row>
@@ -31328,12 +31334,12 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>SIRI</t>
+          <t>CATO</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Sirius XM Holdings Inc.</t>
+          <t>The Cato Corporation</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
@@ -31343,11 +31349,11 @@
       </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Communication </t>
+          <t>Consumer Discr</t>
         </is>
       </c>
       <c r="F32" s="18" t="n">
-        <v>9543175168</v>
+        <v>66662584</v>
       </c>
       <c r="G32" s="19" t="inlineStr">
         <is>
@@ -31355,40 +31361,40 @@
         </is>
       </c>
       <c r="H32" s="20" t="n">
-        <v>7.839</v>
+        <v>134.466</v>
       </c>
       <c r="I32" s="20" t="n">
-        <v>12.0127125</v>
+        <v>2.916295653927599</v>
       </c>
       <c r="J32" s="22" t="n">
-        <v>12.80212302889506</v>
+        <v>34.35404370485792</v>
       </c>
       <c r="K32" s="22" t="n">
-        <v>10.57658645741083</v>
+        <v>6.90904715732555</v>
       </c>
       <c r="L32" s="22" t="n">
-        <v>25.19519869479081</v>
+        <v>0.39782078028546</v>
       </c>
       <c r="M32" s="20" t="n">
-        <v>4.4736355226642</v>
+        <v>29.52748942714341</v>
       </c>
       <c r="N32" s="22" t="n">
-        <v>37.51723087267589</v>
+        <v>6.521741571708831</v>
       </c>
       <c r="O32" s="18" t="n">
         <v>2</v>
       </c>
       <c r="P32" s="20" t="n">
-        <v>0.6308860972502057</v>
+        <v>0.9920879293908172</v>
       </c>
       <c r="Q32" s="15" t="inlineStr">
         <is>
-          <t>Sirius XM (76%)</t>
+          <t>Reportable Segments Re (100%)</t>
         </is>
       </c>
       <c r="R32" s="17" t="inlineStr">
         <is>
-          <t>Sirius XM 76%; Pandora And Off Platform 24%</t>
+          <t>Reportable Segments Retail 100%; Reportable Segments Credit 0%</t>
         </is>
       </c>
       <c r="S32" s="18" t="n">
@@ -31397,7 +31403,7 @@
       <c r="T32" s="17" t="n"/>
       <c r="U32" s="15" t="inlineStr">
         <is>
-          <t>Pandora And Off Plat -0%</t>
+          <t>Reportable Segments  +1%</t>
         </is>
       </c>
     </row>
@@ -31407,12 +31413,12 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>SIEB</t>
+          <t>SIRI</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Siebert Financial Corp.</t>
+          <t>Sirius XM Holdings Inc.</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -31422,58 +31428,52 @@
       </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t xml:space="preserve">Communication </t>
         </is>
       </c>
       <c r="F33" s="18" t="n">
-        <v>69599592</v>
+        <v>9543175168</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
           <t>UNRESEARCHED</t>
         </is>
       </c>
-      <c r="H33" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="I33" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J33" s="21" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="H33" s="20" t="n">
+        <v>7.839</v>
+      </c>
+      <c r="I33" s="20" t="n">
+        <v>12.0127125</v>
+      </c>
+      <c r="J33" s="22" t="n">
+        <v>12.80212302889506</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>5.17888936540735</v>
+        <v>10.57658645741083</v>
       </c>
       <c r="L33" s="22" t="n">
-        <v>7.23199371130981</v>
+        <v>25.19519869479081</v>
       </c>
       <c r="M33" s="20" t="n">
-        <v>-1.897588315217392</v>
+        <v>4.4736355226642</v>
       </c>
       <c r="N33" s="22" t="n">
-        <v>-64.87603317998357</v>
+        <v>37.51723087267589</v>
       </c>
       <c r="O33" s="18" t="n">
         <v>2</v>
       </c>
       <c r="P33" s="20" t="n">
-        <v>0.9865046689171856</v>
+        <v>0.6308860972502057</v>
       </c>
       <c r="Q33" s="15" t="inlineStr">
         <is>
-          <t>Financial Services (99%)</t>
+          <t>Sirius XM (76%)</t>
         </is>
       </c>
       <c r="R33" s="17" t="inlineStr">
         <is>
-          <t>Financial Services 99%; Media Sports And Entertainment 1%</t>
+          <t>Sirius XM 76%; Pandora And Off Platform 24%</t>
         </is>
       </c>
       <c r="S33" s="18" t="n">
@@ -31482,7 +31482,7 @@
       <c r="T33" s="17" t="n"/>
       <c r="U33" s="15" t="inlineStr">
         <is>
-          <t>Financial Services +11%</t>
+          <t>Pandora And Off Plat -0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Meaningful worksheet tab colours + cover legends
New shared tab_colors.py drives tab-strip colouring across every
navigation book so a 50-70 tab workbook encodes structure at a glance:
- Country books (top_n, country_archetype, inflection, OTC): tabs
  coloured by region (DM North America blue, W Europe green, EM Asia
  amber, LatAm burnt-orange, ...) via region_map, so same-region sheets
  cluster in the strip.
- Archetype books (archetype, OTC archetype, segment detail): tabs
  coloured by archetype family (deep-value/quality/inflection/growth/
  capital/lynch/segment/contrarian) — all 69 archetypes mapped.
- Cover/Density/aggregate roll-up tabs get a dark slate so navigation
  sheets stand apart from content.
Each cover carries a compact colour legend (swatch + label) in the
previously-empty right-side columns.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/segment_detail_book.xlsx
+++ b/segment_detail_book.xlsx
@@ -536,6 +536,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF1B2430"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -816,6 +817,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF4A5568"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -27521,6 +27523,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF3949AB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -33372,6 +33375,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF3949AB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -39241,6 +39245,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF3949AB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -45020,6 +45025,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF3949AB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>